<commit_message>
Attach hosted assessments and second-year revision tests to lesson plans
</commit_message>
<xml_diff>
--- a/frontend/templates/lesson-topics-template.xlsx
+++ b/frontend/templates/lesson-topics-template.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Lesson topics" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lesson topics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Lesson topics'!$A$1:$H$3</definedName>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -436,6 +436,7 @@
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="32" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="55" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -479,6 +480,11 @@
           <t>materials</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>test_url</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -494,6 +500,8 @@
           <t>lesson</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
         <v>90</v>
       </c>
@@ -502,6 +510,8 @@
           <t>Noun classification</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -535,12 +545,41 @@
           <t>Parts of Speech; Noun; Article</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Revision Test 1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>revision</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="n">
+        <v>90</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Second-year speaking revision</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H3"/>
   <dataValidations count="1">
     <dataValidation sqref="C2:C121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"lesson,test,credit,exam,imt,extra"</formula1>
+      <formula1>"lesson,test,credit,exam,revision,imt,extra"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>